<commit_message>
docs: add Phase 1A golden output handoff
</commit_message>
<xml_diff>
--- a/outputs/phase-1a-golden/GT-07-GT-09-working.xlsx
+++ b/outputs/phase-1a-golden/GT-07-GT-09-working.xlsx
@@ -1496,7 +1496,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="beJgpJEiG9tPkj3toE1fz44usERRtxD4RAvcSfVDb5LzWx7iAx6/tq42/8S8lkk3S3LfDeUjEWK73lZNmXfm2w==" saltValue="TnCR3/lh7JIm/lTXzHlnUw==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="H7o7+25f8CJ6Fz6OQgnSfV0kB3uukGZlGfjRk/VDFpaBpzrprfMwLgxbp2Pe+cRm08e4NRH499fzb7ZLZRhKsA==" saltValue="kwKNMf8S3uLRaV/X6RPlYA==" spinCount="100000"/>
   <autoFilter ref="A6:B16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1607,7 +1607,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="PW5D1+uaGuHPkfZKp1GqSr2cKkh2yLbfcGRQsRUYabBmRpMq+vHvJoPmiDMv/xgJ3FvWwzuvgyQydCWtD+l6Iw==" saltValue="oeB6KiQTo5NONV/Qdn8fng==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="CefCG+BjQXYHQlWbb5d7Z4HN8TL0Z66wPXrmlq9DV0jvReu2kF4DTEIBq/n3vemNDQnj34dXHm5MdudlA4N1KA==" saltValue="IdyLDZyuks7JQhfpDFz46w==" spinCount="100000"/>
   <autoFilter ref="A6:E7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1787,7 +1787,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="nRk4e4GdHef9Dq2Un5hcNBjAheyKSHUTVTKzFaYirdLeGoU0DZUYgQzNOwrRSuJRxYA9WC9wgSQF2O9OEeKZxA==" saltValue="aXXtKR56SdHpv0t8i5ilkg==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="zNlEApp97f2qMFFMoWd2aLfbMEIUarZx4qY0pjGS2hyTPV3uEprTB8nS0dWzZKg1CxNH/ZEleN5z3KfHtGB2OA==" saltValue="O2iYgsYiHKMSpSpx1rgMkw==" spinCount="100000"/>
   <autoFilter ref="A6:Y7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2294,7 +2294,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="lyuF//HvHY7PtnICSFPTXCZ/cExztkJf4hWvkst3ISqIQ3bItW/giNnsFteYHlCKAkYyBl37Jl3RmHzDlhrKFg==" saltValue="2kl+AtZxiYt9oN+JeY4BXw==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="hnebfYO5SP/Xu4gYafZZG4EDOjYKgBDDB/Wz7N8XbC+DhbRIyVS3BSzph6GTn6on7JH3jD7+yRA2+N0gGxtsow==" saltValue="qKhroT3udH9wk7qo0E1Adg==" spinCount="100000"/>
   <autoFilter ref="A6:Q14"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2441,7 +2441,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="U4k6L5gEI0NurdxNKtSbNmbhrvDxoVI53btZV2Q9Xka0TD/D4LmcJ1IDP1N9bTFHDlSCJmTboOouxgFa/e0B1w==" saltValue="GjogTuKcJ676iwiM2FyZZA==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="yR3QNWr05xqtNfmpkLmYT9UkvNUrz0nuQKmpzVkdxFAhPMQwlEB+6eW240N0JFxw7l+snTbqx8xB7pQFACzweQ==" saltValue="xu+D1snvep/dWlIzJ/4e9w==" spinCount="100000"/>
   <autoFilter ref="A6:S7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2615,7 +2615,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="N6Hr+UZupo178aXbcJEdTri6bPi8oLx39qpWiwfkVBX72RrPhbZLaOJt5TKiOPsB4PQALP+guwGX9+Ew7MQAVQ==" saltValue="We+QYkKFfdYV2ctkUZzelg==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="PHenqI9RBU3Og4dKNGT+k1QzfohOB1Kv6CArNH7sdYLNeIakD+Mwu/z7jThVo2pFliyI2rDbQ5qbKUDf5y9AXw==" saltValue="bGSWp8iQjvsx3BDwkxCdUQ==" spinCount="100000"/>
   <autoFilter ref="A6:P8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2733,7 +2733,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="29dUHBkoHwmibzqVcUdbNIjorGjsvJkKhnjLWQiVEMuEGg3uwLkS6RJ0htPcv3Zag+ExPSejjNyqM/iX6AF72w==" saltValue="hrhVhZ6nrqdOziTu8Vw1XA==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="5VnRowRKZLMur9SNJ0soweWyLfU4b1URWIyE7F6vUS+QGr/IQqyCUZv83YWk7v5aaJK/7y0Nkdh7ALWNWq1k4w==" saltValue="SJ2qeVVUZr0H90VKNRoU9A==" spinCount="100000"/>
   <autoFilter ref="A6:J8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2840,7 +2840,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="PVsDMzkOLUkL5XLpSjPuvScI0Tlr+7zvbEzwrfRHI7qVtuqKR1A73NEABx9LLsyxMhCg/fCNNKgsMxcfP4SwPQ==" saltValue="6PwqE85iVi3gIclK8pVI6A==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="hesVz2VVGvq1KAVnQsZvk2NHzD3ftMEXjzOE4Yuo9y7NulF3y16Kth4xGXOaIdhaxuHqX7Evb3ESsln+oNmPXw==" saltValue="2Z9KGNjVsb7EPMutIaQjXQ==" spinCount="100000"/>
   <autoFilter ref="A6:M7"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2976,7 +2976,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="GC3y3Svb8Xu6HtFVJUB3yDmtUfBpwYQqD6n+DlehV/dpTFtsPz8AXUpMv6pD84wyVL2BM9JmQM1hxXbKJ2u2iA==" saltValue="2KvHK9YUt+HpKDdX6C4tMA==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="fFFz2TEftIHvAFXREyFrP3ctxNAkyXMMwmRLgzAZwfxR+yz05bH+7Bx2xyE2X4scPDimAUvQjuB9ybM4n/XCpA==" saltValue="gDC5I4DE4y6xybiMr09VIg==" spinCount="100000"/>
   <autoFilter ref="A6:L8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>